<commit_message>
Altera links da planilha de TradingView para Investing
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/data/planilha_referencia.xlsx
+++ b/data/planilha_referencia.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillherme\Desktop\Alura\Projeto_macro_tdw\data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Guillherme\Desktop\Alura\smc_lab\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6D50456F-154F-492B-8240-E7B354DB5472}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{67DCA523-979E-4B4E-BD15-556053EF4F45}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-17400" yWindow="-14250" windowWidth="21600" windowHeight="13230" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-49035" yWindow="-16320" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -214,13 +214,13 @@
     <t>Petrobras ADR - Petroleo Brasileiro SA</t>
   </si>
   <si>
-    <t>https://br.tradingview.com/symbols/NYSE-PBR/</t>
-  </si>
-  <si>
-    <t>https://br.tradingview.com/symbols/NYSE-VALE/</t>
-  </si>
-  <si>
-    <t>https://br.tradingview.com/symbols/AMEX-EWZ/</t>
+    <t>https://br.investing.com/equities/petroleo-bras</t>
+  </si>
+  <si>
+    <t>https://br.investing.com/equities/vale-s.a.--americ</t>
+  </si>
+  <si>
+    <t>https://br.investing.com/etfs/ishares-brazil-index</t>
   </si>
 </sst>
 </file>

</xml_diff>